<commit_message>
🛠️ fixed minor errors
</commit_message>
<xml_diff>
--- a/data/Dataset_SL.xlsx
+++ b/data/Dataset_SL.xlsx
@@ -1,20 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28623"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://politoit-my.sharepoint.com/personal/giulio_barletta_polito_it/Documents/Documents/Università/PhD/CementBOpt/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="9" documentId="11_4454EE4B9AAF07C4BD8723E31A37C45507577391" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7B238811-76D1-4047-847D-E5525D40D18E}"/>
+  <xr:revisionPtr revIDLastSave="5" documentId="11_DADD474F729403B6E3A6B9F432B7CA5597D8263D" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B41CC62C-CCB5-45E9-9EF4-18A2AE1B9302}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Datasheet" sheetId="1" r:id="rId1"/>
-    <sheet name="Solubility" sheetId="3" r:id="rId2"/>
+    <sheet name="Solubility" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -864,13 +864,6 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:J23"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="10" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="16.77734375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="23.44140625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="10.109375" bestFit="1" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A1" s="26" t="s">
@@ -1416,7 +1409,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="B1:I14"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>

</xml_diff>